<commit_message>
commit products (cam, phone, smartwatch, tablet)
</commit_message>
<xml_diff>
--- a/backend/data/raw/Aduong data - key moni ear.xlsx
+++ b/backend/data/raw/Aduong data - key moni ear.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/GROUP_10_TOPIC_10_SEMANTIC_SEARCH/backend/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVPC\Documents\tl kì 2\2-Advanced Databases\project\GROUP_10_TOPIC_10_SEMANTIC_SEARCH\backend\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0EBCD7B-2C9B-4EF7-8364-D02480FB472A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19C2401-1F20-425B-A86C-775BE04DA395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
updated raw data for kibo, mouse, earfons
</commit_message>
<xml_diff>
--- a/backend/data/raw/Aduong data - key moni ear.xlsx
+++ b/backend/data/raw/Aduong data - key moni ear.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVPC\Documents\tl kì 2\2-Advanced Databases\project\GROUP_10_TOPIC_10_SEMANTIC_SEARCH\backend\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/GROUP_10_TOPIC_10_SEMANTIC_SEARCH/backend/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19C2401-1F20-425B-A86C-775BE04DA395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="292" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA86AC88-86B7-4076-9D81-38621EE0BC97}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="123">
   <si>
     <t xml:space="preserve">category_id </t>
   </si>
@@ -58,9 +58,6 @@
   </si>
   <si>
     <t>budget_id</t>
-  </si>
-  <si>
-    <t>budget id: 1 = low, 2 = mid, 3 = lux</t>
   </si>
   <si>
     <t>Bàn Phím Có Dây Logitech K120</t>
@@ -72,6 +69,335 @@
     <t>Bàn Phím Có Dây Logitech K120 là dòng bàn phím máy tính phổ thông đến từ thương hiệu Logitech (Thụy Sỹ). Đây là lựa chọn hàng đầu cho nhân viên văn phòng, học sinh, sinh viên hoặc các đơn vị cần trang bị máy tính số lượng lớn với chi phí tiết kiệm. Sản phẩm phù hợp cho các nhu cầu nhập liệu, soạn thảo văn bản dài, học tập và giải trí cơ bản.
 Với thiết kế Full-size 104 phím đầy đủ phím số, người dùng có thể thao tác tính toán và làm việc một cách nhanh chóng. Bàn phím có kết nối dây cắm USB dài 1.5m đảm bảo đường truyền ổn định, không lo độ trễ hay hết pin. Điểm nổi bật nhất là tính năng chống nước đổ tràn, giúp bảo vệ linh kiện nếu lỡ tay làm đổ nước khi đang làm việc.
 Sản phẩm có kiểu dáng thanh lịch, mỏng nhẹ với độ cao chỉ 1.35cm và trọng lượng 550g, cực kỳ linh hoạt để mang theo trong balo. Phím bấm bằng nhựa cao cấp bền bỉ, mang lại cảm giác gõ êm ái và thiết kế cứng cáp giúp tăng tuổi thọ sử dụng lâu dài.</t>
+  </si>
+  <si>
+    <t>Bàn Phím Có Dây Gaming Rapoo V50S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rapoo </t>
+  </si>
+  <si>
+    <t>Bàn Phím Bluetooth Dareu LK160D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dareu </t>
+  </si>
+  <si>
+    <t>Bàn phím có dây Gaming Rapoo V50S là dòng sản phẩm bàn phím giả cơ tiêu biểu trong phân khúc phổ thông của thương hiệu Rapoo. Đây là sự lựa chọn hàng đầu cho những người dùng muốn tìm kiếm một thiết bị ngoại vi có thiết kế năng động, bền bỉ và thẩm mỹ cao mà không cần đầu tư quá nhiều chi phí như các dòng phím cơ cao cấp.
+Sản phẩm được thiết kế hướng đến đối tượng là học sinh, sinh viên và game thủ mới bắt đầu, cần một chiếc bàn phím đa năng phục vụ cho cả việc học tập trên giảng đường lẫn giải trí tại nhà. Với trọng lượng chỉ 550g và kích thước gọn nhẹ, bàn phím giải quyết tốt nhu cầu di động, giúp người dùng dễ dàng mang theo trong balo để làm việc tại quán cafe hoặc học nhóm. Bố cục đầy đủ 104 phím đảm bảo hiệu suất nhập liệu văn bản chính xác cho dân văn phòng, đồng thời đáp ứng tốt các thao tác tổ hợp phím phức tạp khi chơi game.
+Về mặt kỹ thuật, Rapoo V50S sử dụng dây cắm USB dài 1m cho kết nối ổn định tuyệt đối với các máy tính chạy hệ điều hành Windows mà không lo về độ trễ hay hết pin. Hệ thống phím được làm từ chất liệu nhựa ABS bền bỉ, chịu được cường độ gõ phím cao trong thời gian dài. Điểm nhấn ấn tượng nhất chính là hệ thống đèn LED RGB đa sắc màu, không chỉ giúp định vị phím rõ ràng trong môi trường thiếu sáng mà còn tăng cường cảm hứng sáng tạo và tạo nên không gian giải trí đậm chất gaming chuyên nghiệp.</t>
+  </si>
+  <si>
+    <t>Bàn phím Bluetooth Dareu LK160D là dòng phím không dây rút gọn (86 phím) phân khúc phổ thông, giải pháp lý tưởng cho dân văn phòng và sinh viên cần làm việc di động trên Windows, macOS hay điện thoại. Với cấu trúc phím cắt kéo (Scissor) mang lại cảm giác gõ êm ái và yên tĩnh, sản phẩm hỗ trợ kết nối linh hoạt qua Bluetooth hoặc đầu thu USB trong phạm vi 10m. Điểm nhấn nổi bật là trọng lượng siêu nhẹ chỉ 398g, cổng sạc Type-C hiện đại cho thời lượng sử dụng bền bỉ tới 175 giờ, giúp tối ưu không gian làm việc nhỏ gọn và tiện lợi khi mang theo ra ngoài.</t>
+  </si>
+  <si>
+    <t>Bàn phím Bluetooth Logitech K380s là dòng bàn phím không dây Compact (79 phím) cao cấp từ Thụy Sỹ, mang thiết kế thanh lịch và gam màu hồng trang nhã. Sản phẩm là lựa chọn hoàn hảo cho dân văn phòng và người dùng sáng tạo cần sự gọn nhẹ để làm việc di động trên Windows, macOS hay máy tính bảng. Với kết nối Bluetooth ổn định trong phạm vi 10m và khả năng tùy chỉnh qua phần mềm Logi Options+, bàn phím giúp tối ưu không gian làm việc nhỏ nhắn. Điểm nhấn nổi bật là trọng lượng chỉ 423g, sử dụng 2 viên pin AAA tiện lợi, mang lại trải nghiệm gõ phím êm ái và bền bỉ suốt thời gian dài.</t>
+  </si>
+  <si>
+    <t>Bàn Phím Bluetooth Logitech K380s</t>
+  </si>
+  <si>
+    <t>Logitech </t>
+  </si>
+  <si>
+    <t>Bàn phím cơ AULA F75</t>
+  </si>
+  <si>
+    <t>AULA</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ AULA F75 là dòng bàn phím cơ Gasket mount cao cấp với layout 80 phím gọn gàng, mang lại trải nghiệm gõ phím cực kỳ êm ái nhờ lót sẵn 5 lớp foam triệt âm. Đây là lựa chọn hàng đầu cho các lập trình viên và game thủ cần sự linh hoạt nhờ khả năng kết nối 3 chế độ: USB Type-C, Bluetooth và Wireless 2.4G ổn định. Sản phẩm sở hữu mạch xuôi cùng tính năng Hotswap 5-pin giúp người dùng dễ dàng tùy biến switch theo sở thích cá nhân. Điểm nhấn ấn tượng là hệ thống LED RGB rực rỡ trên Plate PC và cấu trúc đệm Gasket bền bỉ, tạo nên sự chuyên nghiệp và cảm hứng làm việc tối đa trong tầm giá 1 triệu đồng.</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ Yunzii C75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yunzii </t>
+  </si>
+  <si>
+    <t>Bàn phím cơ Yunzii C75 Cake Meow là dòng phím 75% (84 phím) cao cấp mang thiết kế tai mèo "siêu cute", phụ kiện đồng bộ hoàn hảo để làm quà tặng cho phái nữ yêu phong cách ngọt ngào. Với cấu trúc Gasket Mount kết hợp foam nhiều lớp và switch Linear êm ái, sản phẩm giải quyết nhu cầu gõ phím yên tĩnh, mượt mà cho các bạn nữ làm văn phòng hoặc sáng tạo nội dung. Điểm nhấn nổi bật là kết nối 3 chế độ linh hoạt, pin khủng 5500 mAh và hệ thống LED RGB South-facing rực rỡ, mang lại trải nghiệm sử dụng tinh tế và bền bỉ trên cả Windows lẫn macOS.</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ Fullsize Weikav NUT108 là dòng phím nhôm CNC nguyên khối cao cấp (108 phím), giải pháp đẳng cấp cho người dùng chuyên nghiệp và các tín đồ custom phím cần sự đầm chắc, sang trọng. Với cơ chế Ball Catch tháo lắp nhanh không dùng ốc và mạch Flexcut 1.2mm, sản phẩm mang lại trải nghiệm gõ HIFI nhún nhảy, êm ái kèm âm thanh tiêu âm cực tốt. Điểm nhấn vượt trội là viên pin khủng 10.000mAh, kết nối 3 chế độ linh hoạt và hệ thống Double Light Bar với LED viền rực rỡ, giúp tối ưu hóa hiệu suất làm việc và thẩm mỹ cho không gian setup hi-end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bàn phím cơ Fullsize Weikav NUT108 </t>
+  </si>
+  <si>
+    <t>Weikav</t>
+  </si>
+  <si>
+    <t>Magic Keyboard cho iPad Pro M4/M5 11 inch</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Bàn phím Apple Magic Keyboard cho iPad Pro 11 inch (M4) là phụ kiện cao cấp biến máy tính bảng thành laptop chuyên nghiệp, mang lại trải nghiệm gõ phím tuyệt vời và chính xác. Sản phẩm là lựa chọn hàng đầu cho doanh nhân và người dùng sáng tạo cần sự mỏng nhẹ, linh hoạt để làm việc hiệu suất cao trên iPadOS mọi lúc mọi nơi. Với kết nối Smart Connector tức thì và tích hợp Trackpad điều khiển con trỏ mượt mà, bàn phím giúp tối ưu hóa các tác vụ đa nhiệm phức tạp. Điểm nhấn nổi bật là thiết kế siêu mỏng, tích hợp đèn nền LED tiện dụng và cổng sạc USB-C riêng biệt, đảm bảo không gian làm việc tối giản và sang trọng.</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ EVO75</t>
+  </si>
+  <si>
+    <t>Evoworks</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ Evoworks Evo75 là dòng phím custom 75% cao cấp với khung nhôm CNC 6063 nguyên khối, mang lại trải nghiệm gõ "đầm" và sang trọng bậc nhất cho các tín đồ công nghệ. Sản phẩm là lựa chọn tối ưu cho lập trình viên và người dùng hi-end cần sự linh hoạt nhờ kết nối 3 chế độ cùng khả năng tùy chỉnh phím qua phần mềm VIA/QMK chuyên nghiệp. Với cấu trúc lò xo cánh bướm (Butterfly Leaf Spring) độc đáo và dung lượng pin khủng 8000mAh, bàn phím giải quyết triệt để nhu cầu về cảm giác gõ đàn hồi và thời gian sử dụng không dây cực dài. Điểm nhấn vượt trội là cơ chế tháo lắp nhanh ball-catch không dùng vít và hệ thống LED mạch xuôi tinh tế, tạo nên một không gian làm việc đẳng cấp và đầy cảm hứng.</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ Datamancer The Machinist là dòng sản phẩm thủ công cao cấp với khung nhôm đúc nguyên khối, mang phong cách cơ khí công nghiệp (Industrial) độc bản và sang trọng. Đây là lựa chọn đẳng cấp dành cho những nhà sưu tầm hoặc người dùng yêu thích vẻ đẹp hoài cổ, muốn tìm kiếm cảm giác gõ khác biệt trên các hệ điều hành Windows, macOS hay Linux. Với switch Cherry MX Blue từ Đức tạo tiếng click đặc trưng như máy đánh chữ cổ điển và bộ keycap bọc kim loại siêu bền, sản phẩm giải quyết hoàn hảo nhu cầu về một thiết bị nhập liệu vừa là tác phẩm nghệ thuật, vừa có độ bền cực cao. Điểm nhấn vượt trội là hệ thống chân đế dạng bánh răng cơ khí, dây cáp bọc vải dù 1.8m chắc chắn và khả năng hỗ trợ phần cứng đa dạng các layout phím, khẳng định vị thế cá nhân trong mọi không gian làm việc.</t>
+  </si>
+  <si>
+    <t>Bàn phím cơ Datamancer The Machinist</t>
+  </si>
+  <si>
+    <t>Datamancer</t>
+  </si>
+  <si>
+    <t>Chuột Có dây Silent Rapoo N1200</t>
+  </si>
+  <si>
+    <t>Chuột có dây Silent Rapoo N1200 là dòng chuột quang văn phòng phân khúc giá rẻ với thiết kế đối xứng lịch lãm, phù hợp cho cả người thuận tay trái và tay phải. Sản phẩm là lựa chọn tối ưu cho học sinh, sinh viên và nhân viên văn phòng cần sự tập trung cao độ nhờ tích hợp công nghệ Silent giúp click chuột êm ái, không gây tiếng ồn khó chịu trong môi trường yên tĩnh. Với độ phân giải 1000 DPI chuẩn xác và dây cắm USB dài 152 cm kết nối ổn định, chuột giải quyết tốt các tác vụ lướt web, soạn thảo văn bản và chỉnh sửa ảnh cơ bản trên Windows. Điểm nhấn nổi bật là trọng lượng siêu nhẹ 85g cùng bánh xe lăn chống trượt bền bỉ, mang lại cảm giác di chuyển mượt mà và tiện lợi cho nhu cầu làm việc hàng ngày.</t>
+  </si>
+  <si>
+    <t>Chuột Không dây Silent Rapoo B2S</t>
+  </si>
+  <si>
+    <t>Chuột không dây Silent Rapoo B2S màu xanh là dòng chuột quang không dây phân khúc phổ thông với thiết kế công thái học đối xứng, phù hợp cho cả người thuận tay trái và tay phải. Sản phẩm là lựa chọn lý tưởng cho sinh viên và nhân viên văn phòng cần sự yên tĩnh tối đa khi làm việc ban đêm hoặc trong môi trường công cộng nhờ tích hợp công nghệ Silent chống ồn. Với độ phân giải 1200 DPI và kết nối đầu thu USB Receiver ổn định trong phạm vi 10m, chuột giải quyết tốt các nhu cầu học tập và thao tác tin học văn phòng hàng ngày trên hệ điều hành Windows. Điểm nhấn nổi bật là trọng lượng siêu nhẹ chỉ 60g, sử dụng một viên pin AA tiện lợi, mang lại cảm giác cầm nắm chắc chắn và tính di động cao cho người dùng năng động.</t>
+  </si>
+  <si>
+    <t>Chuột Không Dây Silent Ugreen MU105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ugreen </t>
+  </si>
+  <si>
+    <t>Chuột không dây Silent Ugreen MU105 màu hồng là dòng chuột quang không dây tối giản với thiết kế bo tròn chắc chắn, mang lại cảm giác cầm nắm êm ái và trang nhã cho không gian làm việc. Sản phẩm là lựa chọn tuyệt vời cho nhân viên văn phòng và người dùng sáng tạo cần độ chính xác cao trên nhiều hệ điều hành như Windows, macOS, Linux hay ChromeOS. Với độ phân giải lên đến 2400 DPI và công nghệ Silent chống ồn, chuột giải quyết tốt các tác vụ chỉnh sửa hình ảnh cơ bản và làm việc yên tĩnh trong môi trường công cộng. Điểm nhấn nổi bật là kết nối đầu thu USB ổn định trong phạm vi 10m, trọng lượng 100g đầm tay và sử dụng một viên pin AA tiện lợi, đảm bảo hiệu suất làm việc mượt mà và bền bỉ.</t>
+  </si>
+  <si>
+    <t>Chuột Không dây Silent Logitech M331</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logitech </t>
+  </si>
+  <si>
+    <t>Chuột không dây Silent Logitech M331 là dòng chuột quang công thái học cao cấp từ Thụy Sĩ, nổi bật với thiết kế dành riêng cho người thuận tay phải mang lại sự thoải mái tối ưu. Đây là lựa chọn hàng đầu cho giới văn phòng và người dùng di động cần sự tập trung nhờ công nghệ Silent Mice giảm đến 90% tiếng ồn khi click trên các hệ điều hành Windows, macOS hay Android. Với độ phân giải 1000 DPI chuẩn xác và kết nối đầu thu Nano ổn định trong phạm vi 10m, chuột giải quyết hoàn hảo nhu cầu làm việc mượt mà trên mọi bề mặt mà không gây tiếng động. Điểm nhấn vượt trội là thời lượng pin cực khủng lên đến 24 tháng chỉ với một viên pin AA, giúp người dùng hoàn toàn yên tâm sử dụng lâu dài và tiết kiệm chi phí.</t>
+  </si>
+  <si>
+    <t>Chuột Có dây Gaming Logitech G102 Gen2 Lightsync</t>
+  </si>
+  <si>
+    <t>Chuột Gaming Logitech G102 Gen2 Lightsync là dòng chuột chơi game có dây huyền thoại phân khúc phổ thông từ Thụy Sĩ, nổi bật với thiết kế đối xứng gọn nhẹ phù hợp cho cả người thuận tay trái lẫn tay phải. Sản phẩm là lựa chọn quốc dân cho các game thủ, đặc biệt là người chơi FPS cần sự linh hoạt trong những cú vẩy chuột tốc độ cao nhờ trọng lượng chỉ 85g và mắt đọc Mercury 8000 DPI chuẩn xác. Với hệ thống đèn LED RGB Lightsync 16.8 triệu màu rực rỡ và 6 nút chức năng có thể lập trình qua Logitech G HUB, chuột giải quyết hoàn hảo nhu cầu cá nhân hóa phong cách và tối ưu hóa thao tác khi chiến game trên Windows. Điểm nhấn vượt trội là dây cáp dài 2.1m cực kỳ bền bỉ và cảm giác bấm tách rời nhạy bén, mang lại hiệu suất gaming chuyên nghiệp với mức giá cực kỳ tiếp cận.</t>
+  </si>
+  <si>
+    <t>Chuột không dây MicroPack MP-V01W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MicroPack </t>
+  </si>
+  <si>
+    <t>Chuột không dây Micropack MP-V01W màu xanh lá là dòng chuột quang công thái học cao cấp từ Hồng Kông, sở hữu thiết kế đứng độc đáo giúp giảm áp lực cổ tay và ngăn ngừa hội chứng ống cổ tay. Sản phẩm là lựa chọn hoàn hảo cho dân văn phòng và người dùng chuyên nghiệp thường xuyên làm việc cường độ cao trên Windows hoặc macOS. Với độ phân giải tối đa 1600 DPI và hệ thống 6 nút bấm chức năng, chuột giải quyết triệt để nhu cầu thao tác nhanh chóng và chính xác trong không gian làm việc hiện đại. Điểm nhấn nổi bật là kết nối không dây 2.4GHz ổn định trong phạm vi 10m, trọng lượng 99g đầm tay và sử dụng một viên pin AA tiện lợi, mang lại trải nghiệm sử dụng khỏe mạnh và bền bỉ trong tầm giá</t>
+  </si>
+  <si>
+    <t>Chuột Có dây Gaming Dareu EM950</t>
+  </si>
+  <si>
+    <t>Chuột Gaming DareU EM901X Ultralight là dòng chuột chơi game có dây siêu nhẹ với thiết kế đối xứng, mang lại sự linh hoạt tối đa cho cả người thuận tay trái lẫn tay phải. Đây là lựa chọn hàng đầu cho các game thủ chuyên nghiệp và người chơi hệ FPS cần tốc độ phản xạ cực nhanh nhờ trọng lượng siêu tối ưu chỉ 53g và cảm biến DareU AIM (PixArt PMW3389) đạt độ nhạy lên đến 18.000 DPI. Với hệ thống chân chuột PTFE mượt mà cùng dây cáp dài 182 cm, sản phẩm giải quyết triệt để nhu cầu di chuột không lực cản và độ trễ trên các hệ điều hành Windows hay macOS. Điểm nhấn vượt trội là khả năng tùy chỉnh qua ứng dụng AIM và tần số phản hồi 1000 Hz, giúp tối ưu hóa từng cú click chuẩn xác trong những trận đấu căng thẳng.</t>
+  </si>
+  <si>
+    <t>Chuột sạc Không dây Gaming Rapoo VT9 Air</t>
+  </si>
+  <si>
+    <t>Chuột gaming Rapoo VT9 Air là dòng chuột không dây siêu nhẹ (59g) với thiết kế vỏ ngoài trong suốt độc lạ, mang lại hiệu suất thi đấu đỉnh cao cho các game thủ chuyên nghiệp. Sản phẩm là lựa chọn hoàn hảo cho người chơi hệ tốc độ cần sự chính xác tuyệt đối nhờ cảm biến PAW3398 đạt 26.000 DPI và tốc độ phản hồi siêu tốc 4000Hz (Polling Rate). Với công nghệ phím bấm C+click đồng nhất và kết nối không dây V+ ổn định, chuột giải quyết triệt để vấn đề độ trễ và mỏi cổ tay trong các trận đấu kéo dài trên Windows. Điểm nhấn vượt trội là viên pin sạc dùng tới 180 tiếng qua cổng Type-C, hệ thống 8 nút bấm đa năng và khả năng di chuyển linh hoạt, giúp tối ưu hóa mọi pha xử lý chớp nhoáng trong thế giới ảo.</t>
+  </si>
+  <si>
+    <t>Chuột Có dây Gaming Razer Basilisk V3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Razer </t>
+  </si>
+  <si>
+    <t>Chuột gaming Razer Basilisk V3 là dòng chuột có dây cao cấp với thiết kế công thái học chuyên dụng cho tay phải, mang lại sự thoải mái tuyệt đối cho game thủ và người làm việc sáng tạo trong thời gian dài. Sản phẩm là lựa chọn hàng đầu cho các tựa game FPS hay MOBA nhờ cảm biến Razer Focus+ 26.000 DPI siêu chính xác và switch quang học Gen 2 phản hồi tức thì. Với nút cuộn HyperScroll thông minh và hệ thống 11 nút bấm có thể lập trình qua Razer Synapse 3, chuột giải quyết hoàn hảo nhu cầu tùy biến sâu và thao tác đa nhiệm phức tạp trên Windows. Điểm nhấn vượt trội là dải đèn LED RGB Chroma 11 vùng rực rỡ, kết hợp cùng chân chuột PTFE mượt mà, giúp tối ưu hóa hiệu suất thi đấu và tạo nên phong cách chuyên nghiệp cho mọi góc máy.</t>
+  </si>
+  <si>
+    <t>Chuột sạc Bluetooth Gaming Razer Basilisk V3 Pro White</t>
+  </si>
+  <si>
+    <t>Chuột gaming Razer Basilisk V3 Pro màu trắng là dòng chuột không dây hi-end với thiết kế công thái học tay phải đẳng cấp, mang lại sự thoải mái tuyệt đối cho game thủ chuyên nghiệp. Sản phẩm là lựa chọn hàng đầu cho các tác vụ chơi game và sáng tạo nhờ cảm biến Focus Pro 30K siêu chính xác cùng switch quang học Gen-3 bền bỉ. Với hệ thống 11 nút bấm có thể lập trình, nút cuộn HyperScroll thông minh và kết nối 3 chế độ linh hoạt, chuột giải quyết triệt để nhu cầu tùy biến sâu và hiệu suất cao trên Windows. Điểm nhấn vượt trội là dải đèn Razer Chroma RGB rực rỡ, thời lượng pin 150 giờ cùng khả năng sạc nhanh qua cổng Type-C, khẳng định vị thế dẫn đầu</t>
+  </si>
+  <si>
+    <t>Tai nghe Có dây AVA+ PC-25</t>
+  </si>
+  <si>
+    <t>AVA+</t>
+  </si>
+  <si>
+    <t>Tai nghe có dây AVA+ PC-25 là dòng tai nghe nhét tai phổ thông sở hữu thiết kế hiện đại, gọn nhẹ với khối lượng chỉ 13.6g, mang lại sự thoải mái tối ưu cho người dùng di động. Sản phẩm là lựa chọn kinh tế cho học sinh, sinh viên và nhân viên văn phòng cần một thiết bị âm thanh ổn định để học tập, họp online hay giải trí trên Android, iOS và Windows. Với Driver 10 mm mạnh mẽ cùng mic thoại tích hợp rõ ràng, tai nghe giải quyết tốt nhu cầu đàm thoại và tái hiện âm thanh chi tiết qua jack cắm 3.5 mm truyền thống. Điểm nhấn nổi bật là độ dài dây 1.16m linh hoạt cùng phím điều khiển vật lý tiện lợi, giúp tối ưu hóa trải nghiệm sử dụng hàng ngày một cách đơn giản và hiệu quả.</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth True Wireless Havit TW941</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Havit </t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth Havit TW941 là mẫu tai nghe True Wireless giá rẻ sở hữu thiết kế trẻ trung, siêu nhẹ chỉ 3g, mang lại cảm giác đeo thoải mái và thanh lịch cho người dùng trẻ. Với Driver 13 mm tiên tiến cùng kết nối Bluetooth 5.3 ổn định, sản phẩm giải quyết tốt nhu cầu nghe nhạc chi tiết và đàm thoại rõ nét trên mọi nền tảng từ iOS, Android đến Windows. Điểm nhấn vượt trội là tính năng Game Mode giảm độ trễ, điều khiển cảm ứng đa năng và tổng thời lượng pin lên đến 21 giờ kèm hộp sạc Type-C tiện lợi. Đây là lựa chọn tối ưu cho học sinh, sinh viên cần một thiết bị âm thanh bền bỉ, hiện đại để học tập và giải trí hàng ngày.</t>
+  </si>
+  <si>
+    <t>Tai nghe Chụp Tai Logitech H111</t>
+  </si>
+  <si>
+    <t>Tai nghe chụp tai Logitech H111 là dòng tai nghe Headset có dây siêu nhẹ từ Thụy Sỹ, sở hữu thiết kế tối giản với trọng lượng chỉ 74g mang lại sự thoải mái tuyệt đối khi đeo cả ngày dài. Sản phẩm là lựa chọn quốc dân cho học sinh, sinh viên và nhân viên văn phòng chuyên dùng để học tập trực tuyến, họp video hoặc đàm thoại trên đa nền tảng như Windows, macOS, iOS và Android. Với công nghệ âm thanh nổi rõ nét và micro xoay 180 độ linh hoạt có khả năng giảm thiểu tiếng ồn, tai nghe giải quyết hoàn hảo nhu cầu giao tiếp chuẩn xác và nghe nhạc cơ bản qua jack cắm 3.5 mm phổ biến. Điểm nhấn vượt trội là dây cáp siêu dài 2.35m cho phép tự do di chuyển trong không gian làm việc và quai đeo tùy chỉnh linh hoạt, đảm bảo sự bền bỉ và tiện dụng tối đa cho người dùng.</t>
+  </si>
+  <si>
+    <t>Tai nghe TWS Alpha Works AW-Curve 200</t>
+  </si>
+  <si>
+    <t>Alpha Works</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth TWS Alpha Works AW-Curve 200 là dòng tai nghe Earbuds không dây cao cấp từ Mỹ, nổi bật với thiết kế công thái học thanh lịch và trọng lượng siêu nhẹ chỉ 3.8g, mang lại cảm giác đeo êm ái suốt ngày dài. Sản phẩm là lựa chọn lý tưởng cho những người yêu âm nhạc và thường xuyên di chuyển nhờ công nghệ âm thanh Hi-Fi trung thực kết hợp cùng Driver 13 mm mạnh mẽ, giúp tái hiện dải âm uy lực và chi tiết. Với hệ thống 4 micro tích hợp công nghệ chống ồn môi trường (ENC), tai nghe giải quyết triệt để nhu cầu đàm thoại rõ nét và nghe nhạc tập trung trên các thiết bị iOS, Android hay Windows. Điểm nhấn vượt trội là khả năng kháng nước IPX4 bền bỉ, kết nối Bluetooth 5.4 tiên tiến cùng tổng thời lượng pin lên đến 20 giờ và tính năng sạc nhanh tiện lợi, sẵn sàng đồng hành cùng bạn trong mọi hoạt động tập luyện hay làm việc hàng ngày.</t>
+  </si>
+  <si>
+    <t>Tai nghe chụp tai Sony MDR-ZX110AP</t>
+  </si>
+  <si>
+    <t>Sony</t>
+  </si>
+  <si>
+    <t>Tai nghe chụp tai Sony MDR-ZX110AP là dòng tai nghe có dây mang phong cách Nhật Bản với thiết kế gọn gàng, sành điệu và khả năng gấp gọn linh hoạt, cực kỳ tiện lợi để bỏ vào balo hay túi xách. Sản phẩm là lựa chọn ưu tiên cho học sinh, sinh viên và người dùng trẻ cần một thiết bị âm thanh bền bỉ, thoải mái để học tập và giải trí trên đa nền tảng như Windows, Android, iOS hay Windows Phone. Với màng loa Dynamic Neodymium 30 mm cùng đệm tai mềm mại, tai nghe giải quyết tốt nhu cầu thưởng thức âm thanh rõ ràng, âm bass trầm ấm mà không gây đau tai khi sử dụng trong thời gian dài qua jack cắm 3.5 mm. Điểm nhấn nổi bật là phần quai đeo tùy chỉnh linh hoạt thêm 4.5 cm, tích hợp mic thoại và phím điều khiển đa năng ngay trên dây dài 1.2 m, giúp tối ưu hóa việc nhận cuộc gọi và chuyển bài hát một cách nhanh chóng.</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth Open-Ear OWS Rezo MuseGo 2</t>
+  </si>
+  <si>
+    <t>Rezo</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth TWS Rezo màu be là dòng tai nghe không dây phân khúc tầm trung sở hữu thiết kế thời thượng và nhỏ gọn với khối lượng chỉ 5g, mang lại cảm giác đeo nhẹ nhàng và tinh tế. Sản phẩm là lựa chọn lý tưởng cho giới trẻ và nhân viên văn phòng cần một thiết bị âm thanh hiện đại, hỗ trợ đàm thoại và giải trí mượt mà trên các hệ điều hành iOS, Android hay Windows. Với Driver 10 mm cùng công nghệ kết nối Bluetooth 6.0 tiên tiến, tai nghe giải quyết tốt nhu cầu nghe nhạc chi tiết và kết nối ổn định trong phạm vi rộng. Điểm nhấn vượt trội là màn hình hiển thị dung lượng pin trực quan trên hộp sạc, tổng thời lượng sử dụng lên đến 22 giờ và hệ thống điều khiển cảm ứng đa năng, giúp tối ưu hóa trải nghiệm sử dụng hàng ngày một cách thông minh và tiện lợi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tai nghe Bluetooth Chụp Tai Baseus Bass 35 Max </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseus </t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth chụp tai Baseus Bass 35 Max là dòng tai nghe không dây hiện đại sở hữu thiết kế sang trọng với đệm tai êm ái, mang lại sự thoải mái tuyệt đối cho người dùng trong những phiên nghe nhạc kéo dài. Sản phẩm là lựa chọn tối ưu cho những người trẻ năng động và dân văn phòng cần sự tập trung cao độ nhờ sự kết hợp giữa công nghệ âm thanh vòm (Surround Sound) và khả năng chống ồn (ENC/Passive Noise Cancellation) trên các hệ điều hành iOS, Android hay Windows. Với Driver tích hợp công nghệ Dynamic Bass Boost mạnh mẽ cùng kết nối Bluetooth 5.3 ổn định, tai nghe giải quyết triệt để nhu cầu thưởng thức âm nhạc chất lượng cao và đàm thoại rõ nét. Điểm nhấn vượt trội là thời lượng pin cực khủng lên tới 50 giờ, khả năng gấp gọn tiện lợi và hỗ trợ tùy chỉnh qua ứng dụng Baseus, đảm bảo trải nghiệm giải trí không gián đoạn suốt nhiều ngày liền.</t>
+  </si>
+  <si>
+    <t>AirPods Max</t>
+  </si>
+  <si>
+    <t>Tai nghe chụp tai AirPods Max (2024) là dòng tai nghe không dây ultra-hi-end từ Apple, gây ấn tượng mạnh với sự chuyển đổi sang cổng sạc USB-C hiện đại và bảng màu trẻ trung như cam, tím, vàng. Sản phẩm là lựa chọn tối thượng cho những tín đồ công nghệ và người dùng chuyên nghiệp trong hệ sinh thái Apple cần một thiết bị âm thanh đẳng cấp, kết hợp giữa thời trang và hiệu suất vượt trội. Với chip H1 mạnh mẽ ở mỗi bên tai cùng công nghệ Adaptive EQ và Spatial Audio (âm thanh không gian), tai nghe giải quyết hoàn hảo nhu cầu thưởng thức âm thanh rạp hát sống động và cá nhân hóa trên iPhone, iPad hay MacBook. Điểm nhấn đặc biệt nằm ở khả năng chống ồn chủ động (ANC) Pro đỉnh cao, chế độ xuyên âm linh hoạt và thiết kế lưới thoáng khí độc đáo giúp giảm áp lực khi đeo lâu, đi kèm thời lượng pin 20 giờ bền bỉ giúp nâng tầm trải nghiệm giải trí lên một tiêu chuẩn mới trong tầm giá 13.190.000₫.</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth chụp tai JBL Tour One M3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JBL </t>
+  </si>
+  <si>
+    <t>Tai nghe chụp tai JBL Tour One M2 màu vàng lấp lánh là dòng tai nghe không dây Hi-End từ Mỹ, sở hữu thiết kế sang trọng và công nghệ âm thanh đỉnh cao, mang lại trải nghiệm giải trí đẳng cấp cho người dùng chuyên nghiệp. Sản phẩm là lựa chọn hàng đầu cho những tín đồ âm nhạc khắt khe nhờ sự kết hợp giữa chất âm JBL Pro Sound mạnh mẽ, chuẩn Hi-Res Audio và codec LDAC truyền tải âm thanh chất lượng cao trên các hệ điều hành iOS, Android hay Windows. Với công nghệ True Adaptive Noise Cancelling tự động điều chỉnh theo môi trường và âm thanh không gian 360 Spatial Sound, tai nghe giải quyết triệt để nhu cầu tĩnh lặng tuyệt đối và không gian âm nhạc sống động như rạp hát. Điểm nhấn vượt trội là thời lượng pin cực khủng lên đến 70 giờ, khả năng kết nối Auracast hiện đại cùng tính năng Smart Talk thông minh, giúp tối ưu hóa việc giao tiếp và thưởng thức âm thanh không gián đoạn trong suốt nhiều ngày liền.</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth True Wireless Bowers &amp; Wilkins Pi7 S2</t>
+  </si>
+  <si>
+    <t>Bowers &amp; Wilkins</t>
+  </si>
+  <si>
+    <t>Tai nghe Bluetooth TWS Bowers &amp; Wilkins Pi5 S2 là dòng tai nghe không dây Hi-end đến từ Anh Quốc, sở hữu thiết kế mang hơi hướng tương lai (futuristic) độc đáo, mang lại vẻ ngoài đẳng cấp và khác biệt cho người sở hữu. Sản phẩm là lựa chọn ưu tiên cho những tín đồ âm thanh khắt khe nhờ sự kết hợp giữa Driver 9.2 mm mạnh mẽ và công nghệ Qualcomm aptX, giúp tái hiện chất âm chi tiết, trung thực trên các nền tảng iOS, Android hay Windows. Với hệ thống chống ồn chủ động (ANC) cùng công nghệ lọc âm DSP tiên tiến, tai nghe giải quyết triệt để nhu cầu thưởng thức âm nhạc yên tĩnh và đàm thoại trong trẻo thông qua 3 micro chống ồn tích hợp. Điểm nhấn vượt trội nằm ở khả năng sạc không dây hiện đại, chuẩn kháng nước bụi IP54 bền bỉ và tổng thời lượng pin lên đến 21 giờ, đảm bảo trải nghiệm giải trí sang trọng và tiện nghi mọi lúc mọi nơi.</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_1.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_2.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_3.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_4.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_5.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_6.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_7.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_8.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_9.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/keyboard/keyboard_10.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_1.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_2.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_3.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_4.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_5.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_6.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_7.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_8.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_9.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/mouse/mouse_10.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_1.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_2.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_3.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_4.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_5.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_6.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_7.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_8.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_9.jpg</t>
+  </si>
+  <si>
+    <t>/backend/data/images/earphones/earphones_10.jpg</t>
   </si>
 </sst>
 </file>
@@ -392,7 +718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -401,12 +727,12 @@
     <col min="5" max="5" width="17.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="15.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="20.5546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="35.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="80.6640625" style="1" customWidth="1"/>
     <col min="9" max="9" width="48.88671875" style="1" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -432,7 +758,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="388.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -443,94 +769,229 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F2" s="1">
         <v>165</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>93</v>
+      </c>
       <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1">
+        <v>285</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="C4" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1">
+        <v>390</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="C5" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="1">
+        <v>730</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="C6" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1050</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1800</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="C8" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2690</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="C9" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="1">
+        <v>8190</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="C10" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="1">
+        <v>4000</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="C11" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="1">
+        <v>18200</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -540,80 +1001,230 @@
       <c r="C12" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="1">
+        <v>95</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="C13" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="1">
+        <v>170</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="C14" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="1">
+        <v>160</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="C15" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="1">
+        <v>340</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="C16" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="1">
+        <v>400</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="C17" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="1">
+        <v>480</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="C18" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="1">
+        <v>560</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="C19" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="1">
+        <v>930</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="C20" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" s="1">
+        <v>1200</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="C21" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="1">
+        <v>3900</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -623,77 +1234,227 @@
       <c r="C22" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F22" s="1">
+        <v>70</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
       <c r="C23" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D23" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F23" s="1">
+        <v>190</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
       <c r="C24" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D24" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F24" s="1">
+        <v>200</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
       <c r="C25" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D25" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="1">
+        <v>390</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
       <c r="C26" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F26" s="1">
+        <v>380</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
       <c r="C27" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F27" s="1">
+        <v>490</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
       <c r="C28" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D28" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" s="1">
+        <v>500</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
       <c r="C29" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F29" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="C30" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F30" s="1">
+        <v>9600</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="C31" s="1">
         <v>3</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="1">
+        <v>11280</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>